<commit_message>
added image url in templete and bulk upload processsing
</commit_message>
<xml_diff>
--- a/assets/products-template.xlsx
+++ b/assets/products-template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>Name</t>
   </si>
@@ -40,6 +40,9 @@
     <t>Low Stock Alert</t>
   </si>
   <si>
+    <t>Image URL</t>
+  </si>
+  <si>
     <t>Example Product</t>
   </si>
   <si>
@@ -50,6 +53,9 @@
   </si>
   <si>
     <t>pcs</t>
+  </si>
+  <si>
+    <t>https://images.unsplash.com/photo-1546069901-ba9599a7e63c</t>
   </si>
 </sst>
 </file>
@@ -426,7 +432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I501"/>
+  <dimension ref="A1:J501"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -438,9 +444,10 @@
     <col min="7" max="7" width="8" customWidth="1"/>
     <col min="8" max="8" width="10" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -468,13 +475,16 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C2">
         <v>100</v>
@@ -486,16 +496,19 @@
         <v>50</v>
       </c>
       <c r="F2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H2">
         <v>8</v>
       </c>
       <c r="I2">
         <v>10</v>
+      </c>
+      <c r="J2" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="6:7" x14ac:dyDescent="0.25"/>

</xml_diff>